<commit_message>
data: archive Inflearn homepage 2026-07-24
</commit_message>
<xml_diff>
--- a/inflearn/output/inflearn_main_2026-07-25.xlsx
+++ b/inflearn/output/inflearn_main_2026-07-25.xlsx
@@ -666,7 +666,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R2" s="6" t="inlineStr">
@@ -742,7 +742,7 @@
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R3" s="6" t="inlineStr">
@@ -781,7 +781,7 @@
         <v>6</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -818,7 +818,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
@@ -894,7 +894,7 @@
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -1422,7 +1422,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-25T07:04:57+09:00</t>
+          <t>2026-07-25T08:36:29+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: archive Inflearn homepage 2026-07-25
</commit_message>
<xml_diff>
--- a/inflearn/output/inflearn_main_2026-07-25.xlsx
+++ b/inflearn/output/inflearn_main_2026-07-25.xlsx
@@ -629,7 +629,7 @@
         <v>8</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R2" s="6" t="inlineStr">
@@ -705,7 +705,7 @@
         <v>0</v>
       </c>
       <c r="I3" s="7" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J3" s="7" t="inlineStr">
         <is>
@@ -742,7 +742,7 @@
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R3" s="6" t="inlineStr">
@@ -781,7 +781,7 @@
         <v>6</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>273</v>
+        <v>277</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -818,7 +818,7 @@
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R4" s="6" t="inlineStr">
@@ -857,7 +857,7 @@
         <v>2</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
@@ -894,7 +894,7 @@
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
@@ -930,10 +930,10 @@
         <v>4.9</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>1270</v>
+        <v>1271</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>9772</v>
+        <v>9773</v>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R6" s="6" t="inlineStr">
@@ -1009,7 +1009,7 @@
         <v>5</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J7" s="7" t="inlineStr">
         <is>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R7" s="6" t="inlineStr">
@@ -1085,7 +1085,7 @@
         <v>424</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>9821</v>
+        <v>9830</v>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R8" s="6" t="inlineStr">
@@ -1161,7 +1161,7 @@
         <v>4</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
@@ -1198,7 +1198,7 @@
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R9" s="6" t="inlineStr">
@@ -1237,7 +1237,7 @@
         <v>0</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R10" s="6" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R11" s="6" t="inlineStr">
@@ -1389,7 +1389,7 @@
         <v>60</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R12" s="6" t="inlineStr">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R13" s="6" t="inlineStr">
@@ -1541,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R14" s="6" t="inlineStr">
@@ -1617,7 +1617,7 @@
         <v>154</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>2560</v>
+        <v>2563</v>
       </c>
       <c r="J15" s="7" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R15" s="6" t="inlineStr">
@@ -1730,7 +1730,7 @@
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R16" s="6" t="inlineStr">
@@ -1766,7 +1766,7 @@
         <v>4.9</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>933</v>
@@ -1806,7 +1806,7 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R17" s="6" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R18" s="6" t="inlineStr">
@@ -1958,7 +1958,7 @@
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R19" s="6" t="inlineStr">
@@ -1997,7 +1997,7 @@
         <v>3020</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>56419</v>
+        <v>56421</v>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R20" s="6" t="inlineStr">
@@ -2073,7 +2073,7 @@
         <v>317</v>
       </c>
       <c r="I21" s="7" t="n">
-        <v>3488</v>
+        <v>3491</v>
       </c>
       <c r="J21" s="7" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R21" s="6" t="inlineStr">
@@ -2144,7 +2144,7 @@
         <v>4.7</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I22" s="2" t="n">
         <v>1031</v>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R22" s="6" t="inlineStr">
@@ -2220,7 +2220,7 @@
         <v>5</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>7996</v>
+        <v>7997</v>
       </c>
       <c r="I23" s="7" t="n">
         <v>122422</v>
@@ -2260,7 +2260,7 @@
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R23" s="6" t="inlineStr">
@@ -2336,7 +2336,7 @@
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R24" s="6" t="inlineStr">
@@ -2412,7 +2412,7 @@
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R25" s="6" t="inlineStr">
@@ -2488,7 +2488,7 @@
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R26" s="6" t="inlineStr">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="Q27" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R27" s="6" t="inlineStr">
@@ -2603,7 +2603,7 @@
         <v>49</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R28" s="6" t="inlineStr">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="Q29" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R29" s="6" t="inlineStr">
@@ -2790,7 +2790,7 @@
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R30" s="6" t="inlineStr">
@@ -2829,7 +2829,7 @@
         <v>1511</v>
       </c>
       <c r="I31" s="7" t="n">
-        <v>15228</v>
+        <v>15229</v>
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R31" s="6" t="inlineStr">
@@ -2902,7 +2902,7 @@
         <v>5</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>841</v>
+        <v>842</v>
       </c>
       <c r="I32" s="2" t="n">
         <v>10654</v>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="Q32" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R32" s="6" t="inlineStr">
@@ -3018,7 +3018,7 @@
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R33" s="6" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R34" s="6" t="inlineStr">
@@ -3133,7 +3133,7 @@
         <v>23</v>
       </c>
       <c r="I35" s="7" t="n">
-        <v>1284</v>
+        <v>1288</v>
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
@@ -3170,7 +3170,7 @@
       </c>
       <c r="Q35" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R35" s="6" t="inlineStr">
@@ -3246,7 +3246,7 @@
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R36" s="6" t="inlineStr">
@@ -3322,7 +3322,7 @@
       </c>
       <c r="Q37" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R37" s="6" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R38" s="6" t="inlineStr">
@@ -3474,7 +3474,7 @@
       </c>
       <c r="Q39" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R39" s="6" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R40" s="6" t="inlineStr">
@@ -3589,7 +3589,7 @@
         <v>2</v>
       </c>
       <c r="I41" s="7" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R41" s="6" t="inlineStr">
@@ -3665,7 +3665,7 @@
         <v>1878</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>39448</v>
+        <v>39450</v>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
@@ -3702,7 +3702,7 @@
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R42" s="6" t="inlineStr">
@@ -3741,7 +3741,7 @@
         <v>675</v>
       </c>
       <c r="I43" s="7" t="n">
-        <v>10825</v>
+        <v>10826</v>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
@@ -3778,7 +3778,7 @@
       </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R43" s="6" t="inlineStr">
@@ -3854,7 +3854,7 @@
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R44" s="6" t="inlineStr">
@@ -3930,7 +3930,7 @@
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R45" s="6" t="inlineStr">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R46" s="6" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="Q47" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R47" s="6" t="inlineStr">
@@ -4158,7 +4158,7 @@
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R48" s="6" t="inlineStr">
@@ -4234,7 +4234,7 @@
       </c>
       <c r="Q49" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R49" s="6" t="inlineStr">
@@ -4273,7 +4273,7 @@
         <v>71</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="Q50" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R50" s="6" t="inlineStr">
@@ -4386,7 +4386,7 @@
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R51" s="6" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R52" s="6" t="inlineStr">
@@ -4538,7 +4538,7 @@
       </c>
       <c r="Q53" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R53" s="6" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R54" s="6" t="inlineStr">
@@ -4653,7 +4653,7 @@
         <v>65</v>
       </c>
       <c r="I55" s="7" t="n">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
@@ -4690,7 +4690,7 @@
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R55" s="6" t="inlineStr">
@@ -4766,7 +4766,7 @@
       </c>
       <c r="Q56" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R56" s="6" t="inlineStr">
@@ -4842,7 +4842,7 @@
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R57" s="6" t="inlineStr">
@@ -4918,7 +4918,7 @@
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R58" s="6" t="inlineStr">
@@ -4994,7 +4994,7 @@
       </c>
       <c r="Q59" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R59" s="6" t="inlineStr">
@@ -5033,7 +5033,7 @@
         <v>440</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>20666</v>
+        <v>20667</v>
       </c>
       <c r="J60" s="2" t="inlineStr">
         <is>
@@ -5070,7 +5070,7 @@
       </c>
       <c r="Q60" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R60" s="6" t="inlineStr">
@@ -5146,7 +5146,7 @@
       </c>
       <c r="Q61" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R61" s="6" t="inlineStr">
@@ -5222,7 +5222,7 @@
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R62" s="6" t="inlineStr">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="Q63" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R63" s="6" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="Q64" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R64" s="6" t="inlineStr">
@@ -5413,7 +5413,7 @@
         <v>26</v>
       </c>
       <c r="I65" s="7" t="n">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="Q65" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R65" s="6" t="inlineStr">
@@ -5526,7 +5526,7 @@
       </c>
       <c r="Q66" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R66" s="6" t="inlineStr">
@@ -5565,7 +5565,7 @@
         <v>16</v>
       </c>
       <c r="I67" s="7" t="n">
-        <v>1006</v>
+        <v>1008</v>
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
@@ -5600,7 +5600,7 @@
       </c>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R67" s="6" t="inlineStr">
@@ -5639,7 +5639,7 @@
         <v>0</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
@@ -5676,7 +5676,7 @@
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R68" s="6" t="inlineStr">
@@ -5752,7 +5752,7 @@
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R69" s="6" t="inlineStr">
@@ -5828,7 +5828,7 @@
       </c>
       <c r="Q70" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R70" s="6" t="inlineStr">
@@ -5904,7 +5904,7 @@
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R71" s="6" t="inlineStr">
@@ -5980,7 +5980,7 @@
       </c>
       <c r="Q72" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R72" s="6" t="inlineStr">
@@ -6056,7 +6056,7 @@
       </c>
       <c r="Q73" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R73" s="6" t="inlineStr">
@@ -6132,7 +6132,7 @@
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R74" s="6" t="inlineStr">
@@ -6171,7 +6171,7 @@
         <v>0</v>
       </c>
       <c r="I75" s="7" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
@@ -6208,7 +6208,7 @@
       </c>
       <c r="Q75" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R75" s="6" t="inlineStr">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="Q76" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R76" s="6" t="inlineStr">
@@ -6360,7 +6360,7 @@
       </c>
       <c r="Q77" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R77" s="6" t="inlineStr">
@@ -6436,7 +6436,7 @@
       </c>
       <c r="Q78" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R78" s="6" t="inlineStr">
@@ -6475,7 +6475,7 @@
         <v>0</v>
       </c>
       <c r="I79" s="7" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
@@ -6512,7 +6512,7 @@
       </c>
       <c r="Q79" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R79" s="6" t="inlineStr">
@@ -6551,7 +6551,7 @@
         <v>174</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>5737</v>
+        <v>5739</v>
       </c>
       <c r="J80" s="2" t="inlineStr">
         <is>
@@ -6588,7 +6588,7 @@
       </c>
       <c r="Q80" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R80" s="6" t="inlineStr">
@@ -6664,7 +6664,7 @@
       </c>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R81" s="6" t="inlineStr">
@@ -6740,7 +6740,7 @@
       </c>
       <c r="Q82" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R82" s="6" t="inlineStr">
@@ -6816,7 +6816,7 @@
       </c>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R83" s="6" t="inlineStr">
@@ -6855,7 +6855,7 @@
         <v>0</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="Q84" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R84" s="6" t="inlineStr">
@@ -6968,7 +6968,7 @@
       </c>
       <c r="Q85" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R85" s="6" t="inlineStr">
@@ -7044,7 +7044,7 @@
       </c>
       <c r="Q86" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R86" s="6" t="inlineStr">
@@ -7120,7 +7120,7 @@
       </c>
       <c r="Q87" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R87" s="6" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="Q88" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R88" s="6" t="inlineStr">
@@ -7272,7 +7272,7 @@
       </c>
       <c r="Q89" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R89" s="6" t="inlineStr">
@@ -7348,7 +7348,7 @@
       </c>
       <c r="Q90" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R90" s="6" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="Q91" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R91" s="6" t="inlineStr">
@@ -7500,7 +7500,7 @@
       </c>
       <c r="Q92" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R92" s="6" t="inlineStr">
@@ -7576,7 +7576,7 @@
       </c>
       <c r="Q93" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R93" s="6" t="inlineStr">
@@ -7652,7 +7652,7 @@
       </c>
       <c r="Q94" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R94" s="6" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="Q95" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R95" s="6" t="inlineStr">
@@ -7767,7 +7767,7 @@
         <v>446</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>6398</v>
+        <v>6399</v>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
@@ -7804,7 +7804,7 @@
       </c>
       <c r="Q96" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R96" s="6" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="Q97" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R97" s="6" t="inlineStr">
@@ -7956,7 +7956,7 @@
       </c>
       <c r="Q98" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R98" s="6" t="inlineStr">
@@ -8032,7 +8032,7 @@
       </c>
       <c r="Q99" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R99" s="6" t="inlineStr">
@@ -8071,7 +8071,7 @@
         <v>291</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>4146</v>
+        <v>4147</v>
       </c>
       <c r="J100" s="2" t="inlineStr">
         <is>
@@ -8108,7 +8108,7 @@
       </c>
       <c r="Q100" s="2" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R100" s="6" t="inlineStr">
@@ -8184,7 +8184,7 @@
       </c>
       <c r="Q101" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
       <c r="R101" s="6" t="inlineStr">
@@ -8346,7 +8346,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-25T08:45:46+09:00</t>
+          <t>2026-07-25T12:39:18+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>